<commit_message>
Performance improvements, json, sql, etc.
</commit_message>
<xml_diff>
--- a/data/sponsors.xlsx
+++ b/data/sponsors.xlsx
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1254" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1255" uniqueCount="294">
   <si>
     <t>category</t>
   </si>
@@ -927,6 +927,9 @@
   </si>
   <si>
     <t>Map Points of Interest</t>
+  </si>
+  <si>
+    <t>ring</t>
   </si>
 </sst>
 </file>
@@ -7003,7 +7006,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -7081,11 +7084,11 @@
         <v>3.59</v>
       </c>
       <c r="G9" s="6">
-        <f t="shared" ref="G9:G21" si="0">ROUND(B9/$D$7*100,2)</f>
+        <f t="shared" ref="G9:G22" si="0">ROUND(B9/$D$7*100,2)</f>
         <v>20.66</v>
       </c>
       <c r="H9" s="6">
-        <f t="shared" ref="H9:H21" si="1">ROUND(C9/$E$7*100,2)</f>
+        <f t="shared" ref="H9:H22" si="1">ROUND(C9/$E$7*100,2)</f>
         <v>45.44</v>
       </c>
       <c r="I9" s="6">
@@ -7127,16 +7130,16 @@
         <v>25.11</v>
       </c>
       <c r="I10" s="6">
-        <f t="shared" ref="I10:I21" si="2">ROUND(D10/$D$7*100,2)</f>
+        <f t="shared" ref="I10:I22" si="2">ROUND(D10/$D$7*100,2)</f>
         <v>17.3</v>
       </c>
       <c r="J10" s="6">
-        <f t="shared" ref="J10:J21" si="3">ROUND(E10/$E$7*100,2)</f>
+        <f t="shared" ref="J10:J22" si="3">ROUND(E10/$E$7*100,2)</f>
         <v>19.53</v>
       </c>
       <c r="K10" s="6"/>
       <c r="L10" t="str">
-        <f t="shared" ref="L10:L21" si="4">"    left: "&amp;G10&amp;", top: "&amp;H10&amp;", width: "&amp;I10&amp;", height: "&amp;J10&amp;","</f>
+        <f t="shared" ref="L10:L22" si="4">"    left: "&amp;G10&amp;", top: "&amp;H10&amp;", width: "&amp;I10&amp;", height: "&amp;J10&amp;","</f>
         <v xml:space="preserve">    left: 14.96, top: 25.11, width: 17.3, height: 19.53,</v>
       </c>
     </row>
@@ -7558,8 +7561,46 @@
         <v xml:space="preserve">    left: 72.12, top: 29.67, width: 13.07, height: 26.23,</v>
       </c>
     </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>293</v>
+      </c>
+      <c r="B22" s="6">
+        <v>7.71</v>
+      </c>
+      <c r="C22" s="6">
+        <v>6.38</v>
+      </c>
+      <c r="D22" s="6">
+        <v>1.91</v>
+      </c>
+      <c r="E22" s="6">
+        <v>2.8</v>
+      </c>
+      <c r="G22" s="6">
+        <f t="shared" si="0"/>
+        <v>56.28</v>
+      </c>
+      <c r="H22" s="6">
+        <f t="shared" si="1"/>
+        <v>34.229999999999997</v>
+      </c>
+      <c r="I22" s="6">
+        <f t="shared" si="2"/>
+        <v>13.94</v>
+      </c>
+      <c r="J22" s="6">
+        <f t="shared" si="3"/>
+        <v>15.02</v>
+      </c>
+      <c r="L22" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve">    left: 56.28, top: 34.23, width: 13.94, height: 15.02,</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Baseline before final vendor load before launch.
</commit_message>
<xml_diff>
--- a/data/sponsors.xlsx
+++ b/data/sponsors.xlsx
@@ -15,12 +15,14 @@
     <sheet name="events" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet4" sheetId="4" r:id="rId2"/>
     <sheet name="sponsors" sheetId="2" r:id="rId3"/>
-    <sheet name="animals" sheetId="3" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="5" r:id="rId4"/>
+    <sheet name="animals" sheetId="3" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="events" localSheetId="0">events!$A$1:$H$123</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -48,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1255" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1532" uniqueCount="468">
   <si>
     <t>category</t>
   </si>
@@ -881,9 +883,6 @@
     <t>floral</t>
   </si>
   <si>
-    <t>sensory</t>
-  </si>
-  <si>
     <t>gate</t>
   </si>
   <si>
@@ -896,9 +895,6 @@
     <t>cattle</t>
   </si>
   <si>
-    <t>horse</t>
-  </si>
-  <si>
     <t>H Pos</t>
   </si>
   <si>
@@ -930,6 +926,534 @@
   </si>
   <si>
     <t>ring</t>
+  </si>
+  <si>
+    <t>Level</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Alpco Recycling</t>
+  </si>
+  <si>
+    <t>Admar</t>
+  </si>
+  <si>
+    <t>Casella Waste Systems</t>
+  </si>
+  <si>
+    <t>Waste and Recycling services</t>
+  </si>
+  <si>
+    <t>Fine Line Landscaping</t>
+  </si>
+  <si>
+    <t>Property Services</t>
+  </si>
+  <si>
+    <t>Blue Ribbon</t>
+  </si>
+  <si>
+    <t>Information Technology and Audio Visual Solutions</t>
+  </si>
+  <si>
+    <t>Local Community Publication</t>
+  </si>
+  <si>
+    <t>Hadley's Fab Weld</t>
+  </si>
+  <si>
+    <t>Mercy Flight Inc</t>
+  </si>
+  <si>
+    <t>Air Ambulance Transport Services</t>
+  </si>
+  <si>
+    <t>OPWDD-NYS</t>
+  </si>
+  <si>
+    <t>Superior Plus Propane</t>
+  </si>
+  <si>
+    <t>Vermigreen</t>
+  </si>
+  <si>
+    <t>Compost and Topsoil</t>
+  </si>
+  <si>
+    <t>Lettering Lounge</t>
+  </si>
+  <si>
+    <t>Cusom signs and Graphics</t>
+  </si>
+  <si>
+    <t>A-Verdi Storage</t>
+  </si>
+  <si>
+    <t>Bobcat of the Fingerlakes</t>
+  </si>
+  <si>
+    <t>Brooke's Enterprises</t>
+  </si>
+  <si>
+    <t>Landscaping Company</t>
+  </si>
+  <si>
+    <t>Eastern Shore Insurance Agency</t>
+  </si>
+  <si>
+    <t>John S. Blazey</t>
+  </si>
+  <si>
+    <t>Kubota Dealer</t>
+  </si>
+  <si>
+    <t>Beverage and Food Processing</t>
+  </si>
+  <si>
+    <t>KM Exavating</t>
+  </si>
+  <si>
+    <t>LaMarti's Auto &amp; Diesel Repair</t>
+  </si>
+  <si>
+    <t>Truck and Auto Repair</t>
+  </si>
+  <si>
+    <t>LandPro</t>
+  </si>
+  <si>
+    <t>Agricultural Equipment</t>
+  </si>
+  <si>
+    <t>Long Construction LLC</t>
+  </si>
+  <si>
+    <t>Lyons National Bank</t>
+  </si>
+  <si>
+    <t>McCarthy Tent and Rentals/Nolans Rentals</t>
+  </si>
+  <si>
+    <t>Party Rentals</t>
+  </si>
+  <si>
+    <t>Morrisey Farms</t>
+  </si>
+  <si>
+    <t>Local Agriculture Production</t>
+  </si>
+  <si>
+    <t>MVP Healthcare</t>
+  </si>
+  <si>
+    <t>Healthcare Services</t>
+  </si>
+  <si>
+    <t>Pace Electronics</t>
+  </si>
+  <si>
+    <t>Pal-Mac Service Center</t>
+  </si>
+  <si>
+    <t>Pepsi</t>
+  </si>
+  <si>
+    <t>Spectrum</t>
+  </si>
+  <si>
+    <t>Internet Services</t>
+  </si>
+  <si>
+    <t>T Mobile</t>
+  </si>
+  <si>
+    <t>Tractor Supply</t>
+  </si>
+  <si>
+    <t>Valpak</t>
+  </si>
+  <si>
+    <t>Advertising and Coupons</t>
+  </si>
+  <si>
+    <t>Wayne County Farm Bureau</t>
+  </si>
+  <si>
+    <t>Agricultural Support</t>
+  </si>
+  <si>
+    <t>Meyers RV</t>
+  </si>
+  <si>
+    <t>Show Sponsor</t>
+  </si>
+  <si>
+    <t>Recreational Vehicles</t>
+  </si>
+  <si>
+    <t>4 Paws Canalside Grooming</t>
+  </si>
+  <si>
+    <t>Pet Grooming Services</t>
+  </si>
+  <si>
+    <t>All American Equipment</t>
+  </si>
+  <si>
+    <t>Farm and Construction Equipment</t>
+  </si>
+  <si>
+    <t>Anna Booth Waffles</t>
+  </si>
+  <si>
+    <t>Sugar Waffles</t>
+  </si>
+  <si>
+    <t>Restaurant</t>
+  </si>
+  <si>
+    <t>Brad Jacobs Masonry</t>
+  </si>
+  <si>
+    <t>Residential and Commercial Masonry</t>
+  </si>
+  <si>
+    <t>Bushhog II Mowing</t>
+  </si>
+  <si>
+    <t>Vegetation Management</t>
+  </si>
+  <si>
+    <t>Carpet Spectrum</t>
+  </si>
+  <si>
+    <t>Flooring Sales and Installation</t>
+  </si>
+  <si>
+    <t>Carter Gray Agency</t>
+  </si>
+  <si>
+    <t>Community Bank</t>
+  </si>
+  <si>
+    <t>Banking Services</t>
+  </si>
+  <si>
+    <t>Glovers Crossing Farms</t>
+  </si>
+  <si>
+    <t>Local Agricultural Production</t>
+  </si>
+  <si>
+    <t>JD Chapman Insurance</t>
+  </si>
+  <si>
+    <t>Jennifer Evans</t>
+  </si>
+  <si>
+    <t>Friend of the Fair</t>
+  </si>
+  <si>
+    <t>JLS Accounting</t>
+  </si>
+  <si>
+    <t>Accounting Services</t>
+  </si>
+  <si>
+    <t>Kevin and Ann Evans</t>
+  </si>
+  <si>
+    <t>Konstantinou's Restaurant</t>
+  </si>
+  <si>
+    <t>L Robbins Photography</t>
+  </si>
+  <si>
+    <t>Photographic Services</t>
+  </si>
+  <si>
+    <t>Lake Beverage</t>
+  </si>
+  <si>
+    <t>Beverage Distributor</t>
+  </si>
+  <si>
+    <t>Long Acre Farms</t>
+  </si>
+  <si>
+    <t>Corn Maze, Winery and More</t>
+  </si>
+  <si>
+    <t>Macedon Auto Center</t>
+  </si>
+  <si>
+    <t>Macedon Collision</t>
+  </si>
+  <si>
+    <t>Morgan McTighe</t>
+  </si>
+  <si>
+    <t>NWE Events</t>
+  </si>
+  <si>
+    <t>Event Coordination Services</t>
+  </si>
+  <si>
+    <t>Agricultural Supplies</t>
+  </si>
+  <si>
+    <t>Quigley's Concrete</t>
+  </si>
+  <si>
+    <t>Concrete Patios and sidewalks</t>
+  </si>
+  <si>
+    <t>Reliant Federal Credit Union</t>
+  </si>
+  <si>
+    <t>Vans Auction Service</t>
+  </si>
+  <si>
+    <t>Auction Services</t>
+  </si>
+  <si>
+    <t>Web Trailer Inc.</t>
+  </si>
+  <si>
+    <t>Trailer Manufacturing and Repair</t>
+  </si>
+  <si>
+    <t>Metal Work Services</t>
+  </si>
+  <si>
+    <t>Custom Sheds and More</t>
+  </si>
+  <si>
+    <t>Construction Equipment</t>
+  </si>
+  <si>
+    <t>Excavation Services</t>
+  </si>
+  <si>
+    <t>Waste Management and Recycling Services</t>
+  </si>
+  <si>
+    <t>Automotive Services</t>
+  </si>
+  <si>
+    <t>Developmental Disability Services</t>
+  </si>
+  <si>
+    <t>Red Ribbon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grand Champion </t>
+  </si>
+  <si>
+    <t>Keurig/Dr. Pepper (Motts)</t>
+  </si>
+  <si>
+    <t>Order</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/a_verdi.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/admar.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/alpco.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/brooksenterprise.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/eastern_shore.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/ny_farm_bureau.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/farm_credit.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/fineline.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/fusion_digital.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/genesee_valley.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/hadleys.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/heritage.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/blazey.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/auto_diesel.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/landpro.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/bankwithlbn-logo.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/long_construction.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/macedon_auto.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/marks.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/mccarthy.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/motts.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/pace.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/pepsico.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/superior_plus.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/tmobile.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/tk_auto.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/tractor_supply.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/vermi_green.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/waste_mgmt.webp</t>
+  </si>
+  <si>
+    <t>Bill Gray's</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/all_american_equipment.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/community_bank.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/lake_beverage.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/bill_grays.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/bobcat.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/casella.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/km_excavating.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/l_robbins.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/lettering_lounge.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/mercy_flight.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/meyers_rv.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/opwdd.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/reliant.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/vans.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/pal_mac_service.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/pine_creek.webp</t>
+  </si>
+  <si>
+    <t>Pine Creek Farm &amp; Feed</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/spectrum.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/valpak.webp</t>
+  </si>
+  <si>
+    <t>JemStar Construction</t>
+  </si>
+  <si>
+    <t>/static/icons/fair.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/konst_rest.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/jemstar.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/chapman.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/brad_jacobs.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/carter_gray.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/long_acre.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/carpet.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/morrisey.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/quigley.webp</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/four_paws.webp</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>/static/icons/sponsor/mvp_health.webp</t>
+  </si>
+  <si>
+    <t>infield</t>
+  </si>
+  <si>
+    <t>weekly</t>
+  </si>
+  <si>
+    <t>barn</t>
   </si>
 </sst>
 </file>
@@ -941,7 +1465,7 @@
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -968,6 +1492,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF222222"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -990,7 +1520,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -998,6 +1528,9 @@
     <xf numFmtId="8" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -7006,7 +7539,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -7016,7 +7549,7 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -7026,33 +7559,33 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
+        <v>281</v>
+      </c>
+      <c r="C5" t="s">
+        <v>282</v>
+      </c>
+      <c r="D5" t="s">
+        <v>284</v>
+      </c>
+      <c r="E5" t="s">
         <v>283</v>
       </c>
-      <c r="C5" t="s">
-        <v>284</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="G5" t="s">
         <v>286</v>
       </c>
-      <c r="E5" t="s">
-        <v>285</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
+        <v>287</v>
+      </c>
+      <c r="I5" t="s">
         <v>288</v>
       </c>
-      <c r="H5" t="s">
+      <c r="J5" t="s">
         <v>289</v>
-      </c>
-      <c r="I5" t="s">
-        <v>290</v>
-      </c>
-      <c r="J5" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -7084,11 +7617,11 @@
         <v>3.59</v>
       </c>
       <c r="G9" s="6">
-        <f t="shared" ref="G9:G22" si="0">ROUND(B9/$D$7*100,2)</f>
+        <f t="shared" ref="G9:G23" si="0">ROUND(B9/$D$7*100,2)</f>
         <v>20.66</v>
       </c>
       <c r="H9" s="6">
-        <f t="shared" ref="H9:H22" si="1">ROUND(C9/$E$7*100,2)</f>
+        <f t="shared" ref="H9:H23" si="1">ROUND(C9/$E$7*100,2)</f>
         <v>45.44</v>
       </c>
       <c r="I9" s="6">
@@ -7130,16 +7663,16 @@
         <v>25.11</v>
       </c>
       <c r="I10" s="6">
-        <f t="shared" ref="I10:I22" si="2">ROUND(D10/$D$7*100,2)</f>
+        <f t="shared" ref="I10:I23" si="2">ROUND(D10/$D$7*100,2)</f>
         <v>17.3</v>
       </c>
       <c r="J10" s="6">
-        <f t="shared" ref="J10:J22" si="3">ROUND(E10/$E$7*100,2)</f>
+        <f t="shared" ref="J10:J23" si="3">ROUND(E10/$E$7*100,2)</f>
         <v>19.53</v>
       </c>
       <c r="K10" s="6"/>
       <c r="L10" t="str">
-        <f t="shared" ref="L10:L22" si="4">"    left: "&amp;G10&amp;", top: "&amp;H10&amp;", width: "&amp;I10&amp;", height: "&amp;J10&amp;","</f>
+        <f t="shared" ref="L10:L23" si="4">"    left: "&amp;G10&amp;", top: "&amp;H10&amp;", width: "&amp;I10&amp;", height: "&amp;J10&amp;","</f>
         <v xml:space="preserve">    left: 14.96, top: 25.11, width: 17.3, height: 19.53,</v>
       </c>
     </row>
@@ -7335,7 +7868,7 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>277</v>
+        <v>466</v>
       </c>
       <c r="B16" s="6">
         <v>5.67</v>
@@ -7373,7 +7906,7 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B17" s="6">
         <v>6.82</v>
@@ -7411,7 +7944,7 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B18" s="6">
         <v>7.94</v>
@@ -7449,7 +7982,7 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B19" s="6">
         <v>8.5399999999999991</v>
@@ -7487,7 +8020,7 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B20" s="6">
         <v>9.73</v>
@@ -7525,7 +8058,7 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>282</v>
+        <v>467</v>
       </c>
       <c r="B21" s="6">
         <v>9.8800000000000008</v>
@@ -7563,39 +8096,76 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="B22" s="6">
-        <v>7.71</v>
+        <v>6.87</v>
       </c>
       <c r="C22" s="6">
-        <v>6.38</v>
+        <v>8.7100000000000009</v>
       </c>
       <c r="D22" s="6">
-        <v>1.91</v>
+        <v>2.9</v>
       </c>
       <c r="E22" s="6">
-        <v>2.8</v>
+        <v>2.16</v>
       </c>
       <c r="G22" s="6">
         <f t="shared" si="0"/>
-        <v>56.28</v>
+        <v>50.15</v>
       </c>
       <c r="H22" s="6">
         <f t="shared" si="1"/>
-        <v>34.229999999999997</v>
+        <v>46.73</v>
       </c>
       <c r="I22" s="6">
         <f t="shared" si="2"/>
-        <v>13.94</v>
+        <v>21.17</v>
       </c>
       <c r="J22" s="6">
         <f t="shared" si="3"/>
-        <v>15.02</v>
+        <v>11.59</v>
       </c>
       <c r="L22" t="str">
         <f t="shared" si="4"/>
-        <v xml:space="preserve">    left: 56.28, top: 34.23, width: 13.94, height: 15.02,</v>
+        <v xml:space="preserve">    left: 50.15, top: 46.73, width: 21.17, height: 11.59,</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>465</v>
+      </c>
+      <c r="B23" s="6">
+        <v>6.87</v>
+      </c>
+      <c r="C23" s="6">
+        <v>5.49</v>
+      </c>
+      <c r="D23" s="6">
+        <v>2.9</v>
+      </c>
+      <c r="E23" s="6">
+        <v>3.14</v>
+      </c>
+      <c r="G23" s="6">
+        <f t="shared" si="0"/>
+        <v>50.15</v>
+      </c>
+      <c r="H23" s="6">
+        <f t="shared" si="1"/>
+        <v>29.45</v>
+      </c>
+      <c r="I23" s="6">
+        <f t="shared" si="2"/>
+        <v>21.17</v>
+      </c>
+      <c r="J23" s="6">
+        <f t="shared" si="3"/>
+        <v>16.850000000000001</v>
+      </c>
+      <c r="L23" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve">    left: 50.15, top: 29.45, width: 21.17, height: 16.85,</v>
       </c>
     </row>
   </sheetData>
@@ -8140,6 +8710,1209 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E80"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="39.28515625" customWidth="1"/>
+    <col min="2" max="2" width="8.140625" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" customWidth="1"/>
+    <col min="4" max="4" width="59.140625" customWidth="1"/>
+    <col min="5" max="5" width="56.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>463</v>
+      </c>
+      <c r="B1" t="s">
+        <v>401</v>
+      </c>
+      <c r="C1" t="s">
+        <v>292</v>
+      </c>
+      <c r="D1" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>294</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>399</v>
+      </c>
+      <c r="D2" t="s">
+        <v>177</v>
+      </c>
+      <c r="E2" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>295</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>300</v>
+      </c>
+      <c r="D3" t="s">
+        <v>175</v>
+      </c>
+      <c r="E3" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>296</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>300</v>
+      </c>
+      <c r="D4" t="s">
+        <v>297</v>
+      </c>
+      <c r="E4" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>191</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>300</v>
+      </c>
+      <c r="D5" t="s">
+        <v>215</v>
+      </c>
+      <c r="E5" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>298</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>300</v>
+      </c>
+      <c r="D6" t="s">
+        <v>299</v>
+      </c>
+      <c r="E6" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>178</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>300</v>
+      </c>
+      <c r="D7" t="s">
+        <v>301</v>
+      </c>
+      <c r="E7" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B8">
+        <v>2</v>
+      </c>
+      <c r="C8" t="s">
+        <v>300</v>
+      </c>
+      <c r="D8" t="s">
+        <v>302</v>
+      </c>
+      <c r="E8" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>303</v>
+      </c>
+      <c r="B9">
+        <v>2</v>
+      </c>
+      <c r="C9" t="s">
+        <v>300</v>
+      </c>
+      <c r="D9" t="s">
+        <v>391</v>
+      </c>
+      <c r="E9" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>196</v>
+      </c>
+      <c r="B10">
+        <v>2</v>
+      </c>
+      <c r="C10" t="s">
+        <v>300</v>
+      </c>
+      <c r="D10" t="s">
+        <v>392</v>
+      </c>
+      <c r="E10" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>304</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>300</v>
+      </c>
+      <c r="D11" t="s">
+        <v>305</v>
+      </c>
+      <c r="E11" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>306</v>
+      </c>
+      <c r="B12">
+        <v>2</v>
+      </c>
+      <c r="C12" t="s">
+        <v>300</v>
+      </c>
+      <c r="D12" t="s">
+        <v>397</v>
+      </c>
+      <c r="E12" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>307</v>
+      </c>
+      <c r="B13">
+        <v>2</v>
+      </c>
+      <c r="C13" t="s">
+        <v>300</v>
+      </c>
+      <c r="D13" t="s">
+        <v>226</v>
+      </c>
+      <c r="E13" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>308</v>
+      </c>
+      <c r="B14">
+        <v>2</v>
+      </c>
+      <c r="C14" t="s">
+        <v>300</v>
+      </c>
+      <c r="D14" t="s">
+        <v>309</v>
+      </c>
+      <c r="E14" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>312</v>
+      </c>
+      <c r="B15">
+        <v>3</v>
+      </c>
+      <c r="C15" t="s">
+        <v>398</v>
+      </c>
+      <c r="D15" t="s">
+        <v>173</v>
+      </c>
+      <c r="E15" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>313</v>
+      </c>
+      <c r="B16">
+        <v>3</v>
+      </c>
+      <c r="C16" t="s">
+        <v>398</v>
+      </c>
+      <c r="D16" t="s">
+        <v>393</v>
+      </c>
+      <c r="E16" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>314</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>398</v>
+      </c>
+      <c r="D17" t="s">
+        <v>315</v>
+      </c>
+      <c r="E17" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>316</v>
+      </c>
+      <c r="B18">
+        <v>3</v>
+      </c>
+      <c r="C18" t="s">
+        <v>398</v>
+      </c>
+      <c r="D18" t="s">
+        <v>214</v>
+      </c>
+      <c r="E18" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>317</v>
+      </c>
+      <c r="B19">
+        <v>3</v>
+      </c>
+      <c r="C19" t="s">
+        <v>398</v>
+      </c>
+      <c r="D19" t="s">
+        <v>318</v>
+      </c>
+      <c r="E19" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>400</v>
+      </c>
+      <c r="B20">
+        <v>3</v>
+      </c>
+      <c r="C20" t="s">
+        <v>398</v>
+      </c>
+      <c r="D20" t="s">
+        <v>319</v>
+      </c>
+      <c r="E20" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>320</v>
+      </c>
+      <c r="B21">
+        <v>3</v>
+      </c>
+      <c r="C21" t="s">
+        <v>398</v>
+      </c>
+      <c r="D21" t="s">
+        <v>394</v>
+      </c>
+      <c r="E21" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>321</v>
+      </c>
+      <c r="B22">
+        <v>3</v>
+      </c>
+      <c r="C22" t="s">
+        <v>398</v>
+      </c>
+      <c r="D22" t="s">
+        <v>322</v>
+      </c>
+      <c r="E22" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>323</v>
+      </c>
+      <c r="B23">
+        <v>3</v>
+      </c>
+      <c r="C23" t="s">
+        <v>398</v>
+      </c>
+      <c r="D23" t="s">
+        <v>324</v>
+      </c>
+      <c r="E23" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>310</v>
+      </c>
+      <c r="B24">
+        <v>3</v>
+      </c>
+      <c r="C24" t="s">
+        <v>398</v>
+      </c>
+      <c r="D24" t="s">
+        <v>311</v>
+      </c>
+      <c r="E24" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>325</v>
+      </c>
+      <c r="B25">
+        <v>3</v>
+      </c>
+      <c r="C25" t="s">
+        <v>398</v>
+      </c>
+      <c r="D25" t="s">
+        <v>222</v>
+      </c>
+      <c r="E25" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>326</v>
+      </c>
+      <c r="B26">
+        <v>3</v>
+      </c>
+      <c r="C26" t="s">
+        <v>398</v>
+      </c>
+      <c r="D26" t="s">
+        <v>362</v>
+      </c>
+      <c r="E26" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>327</v>
+      </c>
+      <c r="B27">
+        <v>3</v>
+      </c>
+      <c r="C27" t="s">
+        <v>398</v>
+      </c>
+      <c r="D27" t="s">
+        <v>328</v>
+      </c>
+      <c r="E27" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>329</v>
+      </c>
+      <c r="B28">
+        <v>3</v>
+      </c>
+      <c r="C28" t="s">
+        <v>398</v>
+      </c>
+      <c r="D28" t="s">
+        <v>330</v>
+      </c>
+      <c r="E28" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>331</v>
+      </c>
+      <c r="B29">
+        <v>3</v>
+      </c>
+      <c r="C29" t="s">
+        <v>398</v>
+      </c>
+      <c r="D29" t="s">
+        <v>332</v>
+      </c>
+      <c r="E29" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>333</v>
+      </c>
+      <c r="B30">
+        <v>3</v>
+      </c>
+      <c r="C30" t="s">
+        <v>398</v>
+      </c>
+      <c r="D30" t="s">
+        <v>233</v>
+      </c>
+      <c r="E30" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>334</v>
+      </c>
+      <c r="B31">
+        <v>3</v>
+      </c>
+      <c r="C31" t="s">
+        <v>398</v>
+      </c>
+      <c r="D31" t="s">
+        <v>210</v>
+      </c>
+      <c r="E31" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>335</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>398</v>
+      </c>
+      <c r="D32" t="s">
+        <v>225</v>
+      </c>
+      <c r="E32" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>336</v>
+      </c>
+      <c r="B33">
+        <v>3</v>
+      </c>
+      <c r="C33" t="s">
+        <v>398</v>
+      </c>
+      <c r="D33" t="s">
+        <v>337</v>
+      </c>
+      <c r="E33" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>338</v>
+      </c>
+      <c r="B34">
+        <v>3</v>
+      </c>
+      <c r="C34" t="s">
+        <v>398</v>
+      </c>
+      <c r="D34" t="s">
+        <v>227</v>
+      </c>
+      <c r="E34" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>205</v>
+      </c>
+      <c r="B35">
+        <v>3</v>
+      </c>
+      <c r="C35" t="s">
+        <v>398</v>
+      </c>
+      <c r="D35" t="s">
+        <v>210</v>
+      </c>
+      <c r="E35" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>339</v>
+      </c>
+      <c r="B36">
+        <v>3</v>
+      </c>
+      <c r="C36" t="s">
+        <v>398</v>
+      </c>
+      <c r="D36" t="s">
+        <v>228</v>
+      </c>
+      <c r="E36" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>340</v>
+      </c>
+      <c r="B37">
+        <v>3</v>
+      </c>
+      <c r="C37" t="s">
+        <v>398</v>
+      </c>
+      <c r="D37" t="s">
+        <v>341</v>
+      </c>
+      <c r="E37" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>342</v>
+      </c>
+      <c r="B38">
+        <v>3</v>
+      </c>
+      <c r="C38" t="s">
+        <v>398</v>
+      </c>
+      <c r="D38" t="s">
+        <v>343</v>
+      </c>
+      <c r="E38" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>347</v>
+      </c>
+      <c r="B39">
+        <v>4</v>
+      </c>
+      <c r="C39" t="s">
+        <v>345</v>
+      </c>
+      <c r="D39" t="s">
+        <v>348</v>
+      </c>
+      <c r="E39" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>349</v>
+      </c>
+      <c r="B40">
+        <v>4</v>
+      </c>
+      <c r="C40" t="s">
+        <v>345</v>
+      </c>
+      <c r="D40" t="s">
+        <v>350</v>
+      </c>
+      <c r="E40" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>351</v>
+      </c>
+      <c r="B41">
+        <v>4</v>
+      </c>
+      <c r="C41" t="s">
+        <v>345</v>
+      </c>
+      <c r="D41" t="s">
+        <v>352</v>
+      </c>
+      <c r="E41" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>431</v>
+      </c>
+      <c r="B42">
+        <v>4</v>
+      </c>
+      <c r="C42" t="s">
+        <v>345</v>
+      </c>
+      <c r="D42" t="s">
+        <v>353</v>
+      </c>
+      <c r="E42" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>354</v>
+      </c>
+      <c r="B43">
+        <v>4</v>
+      </c>
+      <c r="C43" t="s">
+        <v>345</v>
+      </c>
+      <c r="D43" t="s">
+        <v>355</v>
+      </c>
+      <c r="E43" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>356</v>
+      </c>
+      <c r="B44">
+        <v>4</v>
+      </c>
+      <c r="C44" t="s">
+        <v>345</v>
+      </c>
+      <c r="D44" t="s">
+        <v>357</v>
+      </c>
+      <c r="E44" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>358</v>
+      </c>
+      <c r="B45">
+        <v>4</v>
+      </c>
+      <c r="C45" t="s">
+        <v>345</v>
+      </c>
+      <c r="D45" t="s">
+        <v>359</v>
+      </c>
+      <c r="E45" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>360</v>
+      </c>
+      <c r="B46">
+        <v>4</v>
+      </c>
+      <c r="C46" t="s">
+        <v>345</v>
+      </c>
+      <c r="D46" t="s">
+        <v>214</v>
+      </c>
+      <c r="E46" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>361</v>
+      </c>
+      <c r="B47">
+        <v>4</v>
+      </c>
+      <c r="C47" t="s">
+        <v>345</v>
+      </c>
+      <c r="D47" t="s">
+        <v>362</v>
+      </c>
+      <c r="E47" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>363</v>
+      </c>
+      <c r="B48">
+        <v>4</v>
+      </c>
+      <c r="C48" t="s">
+        <v>345</v>
+      </c>
+      <c r="D48" t="s">
+        <v>364</v>
+      </c>
+      <c r="E48" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>365</v>
+      </c>
+      <c r="B49">
+        <v>4</v>
+      </c>
+      <c r="C49" t="s">
+        <v>345</v>
+      </c>
+      <c r="D49" t="s">
+        <v>214</v>
+      </c>
+      <c r="E49" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>451</v>
+      </c>
+      <c r="B50">
+        <v>4</v>
+      </c>
+      <c r="C50" t="s">
+        <v>345</v>
+      </c>
+      <c r="D50" t="s">
+        <v>222</v>
+      </c>
+      <c r="E50" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>366</v>
+      </c>
+      <c r="B51">
+        <v>4</v>
+      </c>
+      <c r="C51" t="s">
+        <v>345</v>
+      </c>
+      <c r="D51" t="s">
+        <v>367</v>
+      </c>
+      <c r="E51" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>368</v>
+      </c>
+      <c r="B52">
+        <v>4</v>
+      </c>
+      <c r="C52" t="s">
+        <v>345</v>
+      </c>
+      <c r="D52" t="s">
+        <v>369</v>
+      </c>
+      <c r="E52" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>370</v>
+      </c>
+      <c r="B53">
+        <v>4</v>
+      </c>
+      <c r="C53" t="s">
+        <v>345</v>
+      </c>
+      <c r="D53" t="s">
+        <v>367</v>
+      </c>
+      <c r="E53" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>371</v>
+      </c>
+      <c r="B54">
+        <v>4</v>
+      </c>
+      <c r="C54" t="s">
+        <v>345</v>
+      </c>
+      <c r="D54" t="s">
+        <v>353</v>
+      </c>
+      <c r="E54" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>372</v>
+      </c>
+      <c r="B55">
+        <v>4</v>
+      </c>
+      <c r="C55" t="s">
+        <v>345</v>
+      </c>
+      <c r="D55" t="s">
+        <v>373</v>
+      </c>
+      <c r="E55" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>374</v>
+      </c>
+      <c r="B56">
+        <v>4</v>
+      </c>
+      <c r="C56" t="s">
+        <v>345</v>
+      </c>
+      <c r="D56" t="s">
+        <v>375</v>
+      </c>
+      <c r="E56" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>376</v>
+      </c>
+      <c r="B57">
+        <v>4</v>
+      </c>
+      <c r="C57" t="s">
+        <v>345</v>
+      </c>
+      <c r="D57" t="s">
+        <v>377</v>
+      </c>
+      <c r="E57" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>378</v>
+      </c>
+      <c r="B58">
+        <v>4</v>
+      </c>
+      <c r="C58" t="s">
+        <v>345</v>
+      </c>
+      <c r="D58" t="s">
+        <v>396</v>
+      </c>
+      <c r="E58" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>379</v>
+      </c>
+      <c r="B59">
+        <v>4</v>
+      </c>
+      <c r="C59" t="s">
+        <v>345</v>
+      </c>
+      <c r="D59" t="s">
+        <v>396</v>
+      </c>
+      <c r="E59" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>199</v>
+      </c>
+      <c r="B60">
+        <v>4</v>
+      </c>
+      <c r="C60" t="s">
+        <v>345</v>
+      </c>
+      <c r="D60" t="s">
+        <v>353</v>
+      </c>
+      <c r="E60" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>344</v>
+      </c>
+      <c r="B61">
+        <v>4</v>
+      </c>
+      <c r="C61" t="s">
+        <v>345</v>
+      </c>
+      <c r="D61" t="s">
+        <v>346</v>
+      </c>
+      <c r="E61" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>380</v>
+      </c>
+      <c r="B62">
+        <v>4</v>
+      </c>
+      <c r="C62" t="s">
+        <v>345</v>
+      </c>
+      <c r="D62" t="s">
+        <v>367</v>
+      </c>
+      <c r="E62" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>381</v>
+      </c>
+      <c r="B63">
+        <v>4</v>
+      </c>
+      <c r="C63" t="s">
+        <v>345</v>
+      </c>
+      <c r="D63" t="s">
+        <v>382</v>
+      </c>
+      <c r="E63" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>448</v>
+      </c>
+      <c r="B64">
+        <v>4</v>
+      </c>
+      <c r="C64" t="s">
+        <v>345</v>
+      </c>
+      <c r="D64" t="s">
+        <v>383</v>
+      </c>
+      <c r="E64" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>384</v>
+      </c>
+      <c r="B65">
+        <v>4</v>
+      </c>
+      <c r="C65" t="s">
+        <v>345</v>
+      </c>
+      <c r="D65" t="s">
+        <v>385</v>
+      </c>
+      <c r="E65" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>386</v>
+      </c>
+      <c r="B66">
+        <v>4</v>
+      </c>
+      <c r="C66" t="s">
+        <v>345</v>
+      </c>
+      <c r="D66" t="s">
+        <v>215</v>
+      </c>
+      <c r="E66" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>387</v>
+      </c>
+      <c r="B67">
+        <v>4</v>
+      </c>
+      <c r="C67" t="s">
+        <v>345</v>
+      </c>
+      <c r="D67" t="s">
+        <v>388</v>
+      </c>
+      <c r="E67" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>185</v>
+      </c>
+      <c r="B68">
+        <v>4</v>
+      </c>
+      <c r="C68" t="s">
+        <v>345</v>
+      </c>
+      <c r="D68" t="s">
+        <v>395</v>
+      </c>
+      <c r="E68" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>389</v>
+      </c>
+      <c r="B69">
+        <v>4</v>
+      </c>
+      <c r="C69" t="s">
+        <v>345</v>
+      </c>
+      <c r="D69" t="s">
+        <v>390</v>
+      </c>
+      <c r="E69" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" s="7"/>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A78" s="7"/>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A79" s="7"/>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A80" s="7"/>
+    </row>
+  </sheetData>
+  <sortState ref="A2:H69">
+    <sortCondition ref="B2:B69"/>
+    <sortCondition ref="A2:A69"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>

</xml_diff>